<commit_message>
Update quiz question hint formats for 4, 6, 8, 9, 11, 12 and update answer for 4 to 입업
</commit_message>
<xml_diff>
--- a/Worldgame_Quiz_Data.xlsx
+++ b/Worldgame_Quiz_Data.xlsx
@@ -459,9 +459,9 @@
     <col width="14.4" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="16.2" customWidth="1" min="6" max="6"/>
+    <col width="12.6" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="16.2" customWidth="1" min="8" max="8"/>
+    <col width="12.6" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -535,7 +535,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>빙하의 침식으로 만들어진 골짜기에 빙하가 없어진 후 바닷물이 들어와서 생긴 해안을 무엇이라고 하나요? (○○ ○○)</t>
+          <t>빙하의 침식으로 만들어진 골짜기에 빙하가 없어진 후 바닷물이 들어와서 생긴 해안을 무엇이라고 하나요? (○○○ 해안)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>인도와 네팔, 중국 등에 걸쳐 있는 산맥으로, 세계에서 가장 높은 에베레스트산이 있는 산맥은 무엇인가요? (○○○○○)</t>
+          <t>인도와 네팔, 중국 등에 걸쳐 있는 산맥으로, 세계에서 가장 높은 에베레스트산이 있는 산맥은 무엇인가요? (○○○○ 산맥)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -676,22 +676,22 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>캐나다와 러시아 등 침엽수가 많은 냉대 기후 지역에서 주로 발달한 산업에는 무엇이 있나요? (○○, ○○ ○○)</t>
+          <t>캐나다와 러시아 등 침엽수가 많은 냉대 기후 지역에서 주로 발달한 산업에는 무엇이 있나요? (○○)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>임업, 펄프 공업</t>
+          <t>입업</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>임업, 펄프 공업, 임업 펄프 공업, 임업과 펄프 공업, 임업, 펄프</t>
+          <t>입업, 임업, 임업, 펄프 공업, 펄프 공업</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>ㅇㅇ, ㅍㅍ ㄱㅇ</t>
+          <t>ㅇㅇ</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>브라질, 페루 등에 걸쳐 흐르는 하천으로, 세계에서 가장 유량이 많은 하천은 무엇인가요? (○○○)</t>
+          <t>브라질, 페루 등에 걸쳐 흐르는 하천으로, 세계에서 가장 유량이 많은 하천은 무엇인가요? (○○○ 강)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>따뜻한 기후 지역의 얕은 바닷속에 사는 산호와 산호충의 뼈 등이 쌓여 이루어진 암초 해안을 무엇이라고 하나요? (○○○ ○○)</t>
+          <t>따뜻한 기후 지역의 얕은 바닷속에 사는 산호와 산호충의 뼈 등이 쌓여 이루어진 암초 해안을 무엇이라고 하나요? (○○○ 해안)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>하천 주변 지역에서 물 위에 지은 가옥을 무엇이라고 하나요? (○○ ○○)</t>
+          <t>하천 주변 지역에서 물 위에 지은 가옥을 무엇이라고 하나요? (○○ 가옥)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>세계에서 가장 면적이 넓은 사막으로, 아프리카의 북부에 있는 사막은 무엇인가요? (○○○ ○○)</t>
+          <t>세계에서 가장 면적이 넓은 사막으로, 아프리카의 북부에 있는 사막은 무엇인가요? (○○○ 사막)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>건조 기후 지역에서 오아시스나 하천의 물을 이용하여 대추야자 및 밀 등을 재배하는 농업을 무엇이라고 하나요? (○○○○ ○○)</t>
+          <t>건조 기후 지역에서 오아시스나 하천의 물을 이용하여 대추야자 및 밀 등을 재배하는 농업을 무엇이라고 하나요? (○○○○ 농업)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: update terrain card t4 answer to '하천' and question to '(○○)'
</commit_message>
<xml_diff>
--- a/Worldgame_Quiz_Data.xlsx
+++ b/Worldgame_Quiz_Data.xlsx
@@ -1678,27 +1678,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>4. 강 (하천 곡류/평야)</t>
+          <t>4. 하천 (강 곡류/평야)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>위 사진이 나타내는 지형은 무엇일까요? (○)</t>
+          <t>위 사진이 나타내는 지형은 무엇일까요? (○○)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>강</t>
+          <t>하천</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>강, 하천, 강물, 곡류</t>
+          <t>하천, 강, 강물, 곡류</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>ㄱ</t>
+          <t>ㅎㅊ</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">

</xml_diff>